<commit_message>
Started working on the mlbb page
</commit_message>
<xml_diff>
--- a/ROSTERXTXESPORTS(1).xlsx
+++ b/ROSTERXTXESPORTS(1).xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesse/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesse/Desktop/Xtremex gaming website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8934D4F-A8EB-654E-B95C-3BB935860772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9979274B-EEC5-1944-9ACD-17F730C583EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1640" yWindow="5940" windowWidth="19420" windowHeight="11020" xr2:uid="{821C8F8A-E1E3-4EC3-B451-0B5D8B83FC2C}"/>
+    <workbookView xWindow="0" yWindow="4980" windowWidth="19420" windowHeight="11020" xr2:uid="{821C8F8A-E1E3-4EC3-B451-0B5D8B83FC2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>NO_</t>
   </si>
@@ -185,13 +185,97 @@
   </si>
   <si>
     <t>+233 53 424 1268</t>
+  </si>
+  <si>
+    <t>Bright Bosu Appiah</t>
+  </si>
+  <si>
+    <t>AlreadyPro</t>
+  </si>
+  <si>
+    <t>GE6902SFBR</t>
+  </si>
+  <si>
+    <t>alreadypro20@gmail.com</t>
+  </si>
+  <si>
+    <t>Aaron Gogo Ashirifi</t>
+  </si>
+  <si>
+    <t>Gogo</t>
+  </si>
+  <si>
+    <t>GE4352SFGAR</t>
+  </si>
+  <si>
+    <t>ashirifiaaron@gmail.com</t>
+  </si>
+  <si>
+    <t>Nyantakyi Barima Agyapong</t>
+  </si>
+  <si>
+    <t>Beast</t>
+  </si>
+  <si>
+    <t>GE1253SFAS</t>
+  </si>
+  <si>
+    <t>nyantakyibarima@gmail.com</t>
+  </si>
+  <si>
+    <t>Emmanuel Lartey</t>
+  </si>
+  <si>
+    <t>Igris</t>
+  </si>
+  <si>
+    <t>GE2780SFGAR</t>
+  </si>
+  <si>
+    <t>emmanuellarteye@gmail.com</t>
+  </si>
+  <si>
+    <t>Jesse-Linden Asare Joseph</t>
+  </si>
+  <si>
+    <t>jesselinden234@gmail.com</t>
+  </si>
+  <si>
+    <t>Emmanuel Kofi Danquah</t>
+  </si>
+  <si>
+    <t>Sunless</t>
+  </si>
+  <si>
+    <t>GE2165SFOR</t>
+  </si>
+  <si>
+    <t>kofidanquah543@gmail.com</t>
+  </si>
+  <si>
+    <t>+233 50 183 0637</t>
+  </si>
+  <si>
+    <t>+233 20 741 7412</t>
+  </si>
+  <si>
+    <t>+233 59 258 2617</t>
+  </si>
+  <si>
+    <t>+233 53 147 1840</t>
+  </si>
+  <si>
+    <t>+233 53 802 9516</t>
+  </si>
+  <si>
+    <t>+233 24 007 7160</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,6 +405,31 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF6AA84F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -355,7 +464,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -415,6 +524,12 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1530,54 +1645,181 @@
       <c r="K54" s="15"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A55" s="5" t="s">
+      <c r="A55" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="24">
         <v>1</v>
       </c>
+      <c r="C55" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D55" s="26"/>
+      <c r="E55" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F55" s="26"/>
+      <c r="G55" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="H55" s="26"/>
+      <c r="I55" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="J55" s="27" t="s">
+        <v>58</v>
+      </c>
       <c r="K55" s="15"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B56" s="2">
+      <c r="A56" s="26"/>
+      <c r="B56" s="24">
         <v>2</v>
       </c>
+      <c r="C56" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D56" s="26"/>
+      <c r="E56" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="F56" s="26"/>
+      <c r="G56" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="H56" s="26"/>
+      <c r="I56" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="J56" s="28" t="s">
+        <v>59</v>
+      </c>
       <c r="K56" s="15"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B57" s="2">
+      <c r="A57" s="26"/>
+      <c r="B57" s="24">
         <v>3</v>
       </c>
+      <c r="C57" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D57" s="26"/>
+      <c r="E57" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F57" s="26"/>
+      <c r="G57" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="H57" s="26"/>
+      <c r="I57" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="J57" s="28" t="s">
+        <v>60</v>
+      </c>
       <c r="K57" s="15"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B58" s="2">
+      <c r="A58" s="26"/>
+      <c r="B58" s="24">
         <v>4</v>
       </c>
+      <c r="C58" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="D58" s="26"/>
+      <c r="E58" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="F58" s="26"/>
+      <c r="G58" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="H58" s="26"/>
+      <c r="I58" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="J58" s="28" t="s">
+        <v>61</v>
+      </c>
       <c r="K58" s="15"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B59" s="2">
+      <c r="A59" s="26"/>
+      <c r="B59" s="24">
         <v>5</v>
       </c>
+      <c r="C59" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="D59" s="26"/>
+      <c r="E59" s="26"/>
+      <c r="F59" s="26"/>
+      <c r="G59" s="26"/>
+      <c r="H59" s="26"/>
+      <c r="I59" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="J59" s="28" t="s">
+        <v>62</v>
+      </c>
       <c r="K59" s="15"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B60" s="2">
+      <c r="A60" s="26"/>
+      <c r="B60" s="24">
         <v>6</v>
       </c>
+      <c r="C60" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D60" s="26"/>
+      <c r="E60" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="F60" s="26"/>
+      <c r="G60" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="H60" s="26"/>
+      <c r="I60" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="J60" s="28" t="s">
+        <v>63</v>
+      </c>
       <c r="K60" s="15"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B61" s="2">
+      <c r="A61" s="26"/>
+      <c r="B61" s="24">
         <v>7</v>
       </c>
+      <c r="C61" s="26"/>
+      <c r="D61" s="26"/>
+      <c r="E61" s="26"/>
+      <c r="F61" s="26"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="26"/>
+      <c r="I61" s="26"/>
+      <c r="J61" s="26"/>
       <c r="K61" s="15"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B62" s="2">
+      <c r="A62" s="26"/>
+      <c r="B62" s="24">
         <v>8</v>
       </c>
+      <c r="C62" s="26"/>
+      <c r="D62" s="26"/>
+      <c r="E62" s="26"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="26"/>
+      <c r="I62" s="26"/>
+      <c r="J62" s="26"/>
       <c r="K62" s="15"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>